<commit_message>
Auto update RUP 2026-08-25 15:49:08
</commit_message>
<xml_diff>
--- a/output/rup/2026/Rekap RUP Tahun 2026 (2026-08-25).xlsx
+++ b/output/rup/2026/Rekap RUP Tahun 2026 (2026-08-25).xlsx
@@ -1596,10 +1596,10 @@
         <v>5082238023</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>5051110023</v>
+        <v>5169025413</v>
       </c>
       <c r="F31" s="3" t="n">
         <v>0</v>
@@ -1608,16 +1608,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>5051110023</v>
+        <v>5169025413</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>-31128000</v>
+        <v>86787390</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>99.38751392872337</v>
+        <v>101.707660869232</v>
       </c>
     </row>
     <row r="32">
@@ -3187,10 +3187,10 @@
         <v>1367194468</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>320865383</v>
+        <v>546608944</v>
       </c>
       <c r="F74" s="3" t="n">
         <v>0</v>
@@ -3199,16 +3199,16 @@
         <v>0</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="I74" s="3" t="n">
-        <v>320865383</v>
+        <v>546608944</v>
       </c>
       <c r="J74" s="3" t="n">
-        <v>-1046329085</v>
+        <v>-820585524</v>
       </c>
       <c r="K74" s="4" t="n">
-        <v>23.46889125944006</v>
+        <v>39.98033614044729</v>
       </c>
     </row>
     <row r="75">
@@ -3372,10 +3372,10 @@
         <v>8905641688</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>7895641688</v>
+        <v>8755641688</v>
       </c>
       <c r="F79" s="3" t="n">
         <v>1</v>
@@ -3384,16 +3384,16 @@
         <v>150000000</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>8045641688</v>
+        <v>8905641688</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>-860000000</v>
+        <v>0</v>
       </c>
       <c r="K79" s="4" t="n">
-        <v>90.3432000732882</v>
+        <v>100</v>
       </c>
     </row>
     <row r="80">

</xml_diff>